<commit_message>
Plant heat balance: station gas preheater fuel counted in the plant heat rate (fuel_consumers, stream 31)
Net heat rate at SRC 5,764 kJ/kWh (guarantee 5,860); power island gross heat rate unchanged. HMB
diagram layout: stream 31 and the preheater burner boundary, stream 19 moved clear of the labels.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TuQPCZMPzEzscTVqEEHFMo
</commit_message>
<xml_diff>
--- a/output/hmb/ALP-HMB-CASES.xlsx
+++ b/output/hmb/ALP-HMB-CASES.xlsx
@@ -457,7 +457,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>engine hmb v1.1.1 | data a6baea26d6584942 | 2026-09-29T02:54:45Z</t>
+          <t>engine hmb v1.1.1 | data b6f4b950c7f3b7e0 | 2026-09-29T03:02:22Z</t>
         </is>
       </c>
     </row>
@@ -1024,31 +1024,31 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>831.37</v>
+        <v>832.17</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>1056.05</v>
+        <v>1058.31</v>
       </c>
       <c r="E16" s="3" t="n">
         <v>961.22</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>634.14</v>
+        <v>635.13</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>981.51</v>
+        <v>983.02</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>826.0599999999999</v>
+        <v>827.33</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>412.22</v>
+        <v>412.86</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>880.33</v>
+        <v>881.16</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>1061.51</v>
+        <v>1063.78</v>
       </c>
     </row>
     <row r="17">
@@ -1063,31 +1063,31 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>5830.85</v>
+        <v>5836.42</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>5735.96</v>
+        <v>5748.24</v>
       </c>
       <c r="E17" s="3" t="n">
         <v>6094.42</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>6194.41</v>
+        <v>6204.01</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>5755.32</v>
+        <v>5764.23</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>5894.38</v>
+        <v>5903.5</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>6942.12</v>
+        <v>6952.83</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>5802.15</v>
+        <v>5807.66</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>5740.47</v>
+        <v>5752.77</v>
       </c>
     </row>
     <row r="18">
@@ -1102,31 +1102,31 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>61.74</v>
+        <v>61.68</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>62.76</v>
+        <v>62.63</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>59.07</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>58.12</v>
+        <v>58.03</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>62.55</v>
+        <v>62.45</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>61.08</v>
+        <v>60.98</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>51.86</v>
+        <v>51.78</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>62.05</v>
+        <v>61.99</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>62.71</v>
+        <v>62.58</v>
       </c>
     </row>
     <row r="19">
@@ -1141,31 +1141,31 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>17.51</v>
+        <v>17.53</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>22.24</v>
+        <v>22.29</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>22.41</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>13.36</v>
+        <v>13.38</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>20.67</v>
+        <v>20.7</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>17.4</v>
+        <v>17.42</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>8.68</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>18.54</v>
+        <v>18.56</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>22.36</v>
+        <v>22.4</v>
       </c>
     </row>
     <row r="20">
@@ -1180,29 +1180,29 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>86054.38</v>
+        <v>86136.46000000001</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>109310.2</v>
+        <v>109544.14</v>
       </c>
       <c r="E20" s="3" t="n"/>
       <c r="F20" s="3" t="n">
-        <v>65639.2</v>
+        <v>65740.92999999999</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>101594.3</v>
+        <v>101751.57</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>85503.95</v>
+        <v>85636.14999999999</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>42668.43</v>
+        <v>42734.28</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>91121.32000000001</v>
+        <v>91207.82000000001</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>109875.38</v>
+        <v>110110.79</v>
       </c>
     </row>
     <row r="21">

</xml_diff>